<commit_message>
Rewrite Sugar News summaries for 2026-09-10
</commit_message>
<xml_diff>
--- a/reports/2026/09/Sugar News 2026-09-09.xlsx
+++ b/reports/2026/09/Sugar News 2026-09-09.xlsx
@@ -481,7 +481,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C8"/>
+  <dimension ref="A1:C7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.25"/>
   <cols>
     <col width="55" customWidth="1" style="2" min="2" max="2"/>
@@ -505,7 +505,7 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="120.8" customHeight="1" s="2">
+    <row r="2" ht="180" customHeight="1" s="2">
       <c r="A2" s="3" t="inlineStr">
         <is>
           <t>印度</t>
@@ -513,16 +513,16 @@
       </c>
       <c r="B2" s="4" t="inlineStr">
         <is>
-          <t>印度糖业相关机构公布糖产量，糖产量增加至0万吨。糖产量增加会提高当期新增可售糖源，缓解供应压力并压制糖价。来源：ChiniMandi（https://www.chinimandi.com/uttar-pradesh-sugar-output-may-stay-near-9-mt-despite-higher-cane-yields/）。影响：利空糖价</t>
+          <t>北方邦2026/27榨季食糖产量预计维持在约900万吨，低于市场此前超过1000万吨的预期；虽然西部甘蔗单产预计至少提高10%，但糖厂辖区甘蔗面积可能减少10万-20万公顷，邦政府临时面积也从上榨季286.1万公顷降至281.3万公顷。产量预期低于市场预估叠加可能提前开榨、压低糖分回收，意味着北方邦新增可售糖源难以明显放大，对印度国内糖价形成支撑。来源：ChiniMandi（https://www.chinimandi.com/uttar-pradesh-sugar-output-may-stay-near-9-mt-despite-higher-cane-yields/）。影响：利多糖价</t>
         </is>
       </c>
       <c r="C2" s="4" t="inlineStr">
         <is>
-          <t>利空：糖产量增加会提高当期新增可售糖源，缓解供应压力并压制糖价。</t>
+          <t>利多：北方邦产量预期低于市场此前超过1000万吨的判断，叠加早榨可能降低糖分回收，限制新增食糖供应并支撑印度国内糖价。</t>
         </is>
       </c>
     </row>
-    <row r="3" ht="119.7" customHeight="1" s="2">
+    <row r="3" ht="180" customHeight="1" s="2">
       <c r="A3" s="3" t="inlineStr">
         <is>
           <t>印度</t>
@@ -530,16 +530,16 @@
       </c>
       <c r="B3" s="4" t="inlineStr">
         <is>
-          <t>印度原糖市场显示原糖价格，糖价上涨13%。印度原糖价格上涨说明当地可售糖源偏紧或采购需求增强，短期支撑现货糖价。来源：ChiniMandi（https://www.chinimandi.com/world-raw-sugar-prices-jump-13-in-august-on-speculative-fund-buying/）。影响：利多糖价</t>
+          <t>马哈拉施特拉邦政府决定将2026/27榨季甘蔗开榨从11月1日提前至10月15日，204家糖厂可提前开机；该邦糖库存约300万吨，可收割甘蔗面积约155万公顷，上榨季产糖约1300万吨。提前开榨可使新糖在Dasara、Navaratra和Diwali节日前后更早进入市场，短期增加供应、压制印度国内糖价；但原文提示甘蔗成熟度不足可能使糖分回收率下降约1.5%，会削弱实际产糖增量。来源：The Times of India（https://timesofindia.indiatimes.com/city/kolhapur/maha-advances-cane-crushing-season-by-15-days-to-ease-sugar-prices-during-festivities/amp_articleshow/133980085.cms）。影响：利空糖价</t>
         </is>
       </c>
       <c r="C3" s="4" t="inlineStr">
         <is>
-          <t>利多：印度原糖价格上涨说明当地可售糖源偏紧或采购需求增强，短期支撑现货糖价。</t>
+          <t>利空：马哈拉施特拉邦提前开榨会使新糖更早进入节日消费市场，增加短期供应并压制国内糖价；回收率下降风险会削弱但不改变短期投放方向。</t>
         </is>
       </c>
     </row>
-    <row r="4" ht="137.3" customHeight="1" s="2">
+    <row r="4" ht="165.35" customHeight="1" s="2">
       <c r="A4" s="3" t="inlineStr">
         <is>
           <t>印度</t>
@@ -547,16 +547,16 @@
       </c>
       <c r="B4" s="4" t="inlineStr">
         <is>
-          <t>印度现货市场显示食糖价格，食糖价格上涨至Rs 18。印度食糖价格上涨说明当地可售糖源偏紧或采购需求增强，短期支撑现货糖价。来源：ChiniMandi（https://www.chinimandi.com/uttar-pradesh-antyodaya-card-holders-to-get-sugar-at-rs-18-per-kg-despite-higher-market-prices/）。影响：利多糖价</t>
+          <t>印度主要产区糖厂出厂价已从近期接近Rs65/kg回落至Rs48-52/kg，使政府推动的100万吨原糖进口计划吸引力下降；港口精炼厂目前承诺进口约26万吨，真正进入国内市场的只有数千吨。国内糖价回落本身反映现货压力增加，但进口糖成本高于国产糖会推迟后续进口到港，减少新增外部供应对国内市场的压制。来源：ChiniMandi（https://www.chinimandi.com/falling-domestic-sugar-prices-weaken-indias-1-mt-import-push/）。影响：中性</t>
         </is>
       </c>
       <c r="C4" s="4" t="inlineStr">
         <is>
-          <t>利多：印度食糖价格上涨说明当地可售糖源偏紧或采购需求增强，短期支撑现货糖价。</t>
+          <t>中性：国内出厂价回落压制现货糖价，但进口利润恶化会削弱100万吨进口计划的执行力度，减少后续进口糖供应增量。</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="163.15" customHeight="1" s="2">
+    <row r="5" ht="180" customHeight="1" s="2">
       <c r="A5" s="3" t="inlineStr">
         <is>
           <t>印度</t>
@@ -564,63 +564,46 @@
       </c>
       <c r="B5" s="4" t="inlineStr">
         <is>
-          <t>印度现货市场显示食糖价格，食糖价格下跌至15天。印度食糖价格下跌说明当地供应压力增加或采购需求转弱，短期压制现货糖价。来源：The Times of India（https://timesofindia.indiatimes.com/city/kolhapur/maha-advances-cane-crushing-season-by-15-days-to-ease-sugar-prices-during-festivities/amp_articleshow/133980085.cms）。影响：中性</t>
+          <t>北方邦公共分配系统将Antyodaya持卡户补贴糖价格维持为Rs18/kg，大诺伊达约7000名持卡户将合并领取7-9月每卡3公斤糖，明显低于当地公开市场约Rs60-75/kg的糖价。该政策通过政府渠道向低收入家庭定向投放少量低价糖，可缓和局部零售端价格压力，但覆盖量有限，难以改变商业市场的供需结构。来源：ChiniMandi（https://www.chinimandi.com/uttar-pradesh-antyodaya-card-holders-to-get-sugar-at-rs-18-per-kg-despite-higher-market-prices/）。影响：中性</t>
         </is>
       </c>
       <c r="C5" s="4" t="inlineStr">
         <is>
-          <t>中性：印度食糖价格下跌说明当地供应压力增加或采购需求转弱，短期压制现货糖价。</t>
+          <t>中性：补贴糖定向投放有助于缓和局部零售价格压力，但数量和覆盖人群有限，对商业市场可售糖供应影响较小。</t>
         </is>
       </c>
     </row>
-    <row r="6" ht="123.55" customHeight="1" s="2">
+    <row r="6" ht="111.45" customHeight="1" s="2">
       <c r="A6" s="3" t="inlineStr">
         <is>
-          <t>印度</t>
+          <t>泰国</t>
         </is>
       </c>
       <c r="B6" s="4" t="inlineStr">
         <is>
-          <t>印度现货市场显示食糖价格，食糖价格为1 mt。印度食糖价格只给出当前报价，未提供前期价格、成交变化或库存变化，现有信息不足以判断供应收紧或转弱。来源：ChiniMandi（https://www.chinimandi.com/falling-domestic-sugar-prices-weaken-indias-1-mt-import-push/）。影响：中性</t>
+          <t>泰国气象局9月9日预报，孔敬、呵叻、猜也蓬、黎府、那空沙旺、甘烹碧、素可泰、彭世洛等主要甘蔗产区预计出现雷阵雨并伴有局地大雨。泰国甘蔗仍处于生长期，降雨补充土壤水分并改善单产形成条件，提高后期甘蔗和食糖供应预期。来源：泰国气象局（https://tmd.go.th/en/forecast/daily）。影响：利空糖价</t>
         </is>
       </c>
       <c r="C6" s="4" t="inlineStr">
         <is>
-          <t>中性：印度食糖价格只给出当前报价，未提供前期价格、成交变化或库存变化，现有信息不足以判断供应收紧或转弱。</t>
+          <t>利空：生长期降雨改善泰国甘蔗主产区墒情，有利于单产恢复并增加后期食糖供应预期。</t>
         </is>
       </c>
     </row>
-    <row r="7" ht="127.4" customHeight="1" s="2">
+    <row r="7" ht="180" customHeight="1" s="2">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>泰国</t>
+          <t>国际糖市</t>
         </is>
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>泰国气象局预报（2026-09-09），孔敬、呵叻、猜也蓬、黎府、那空沙旺、甘烹碧、素可泰、彭世洛等等主要甘蔗产区预计出现雷阵雨并伴有局地大雨。当前处于甘蔗生长阶段，强降雨、雷阵雨以及预报大雨均有利于补充产区土壤水分，促进甘蔗生长和单产形成，提高后期甘蔗及食糖产量预期。来源：泰国气象局（https://tmd.go.th/en/forecast/daily）。影响：利空糖价</t>
+          <t>国际糖业组织8月市场报告显示，10月原糖期货从月初约15美分/磅升至8月31日17.8美分/磅，ISA日均原糖价8月均值17.4美分/磅、环比上涨2.0美分或13%，白糖指数均值升至513美元/吨、环比上涨47美元或10%。上涨主要来自投机基金持仓由接近12万手净空转为9月1日超过13.2万手净多，相当于1270万吨糖的持仓摆动，短线推高原糖风险溢价；但报告同时提示主要出口来源仍有较大可出口量、进口需求偏弱，价格追高后存在回落风险。来源：ChiniMandi（https://www.chinimandi.com/world-raw-sugar-prices-jump-13-in-august-on-speculative-fund-buying/）。影响：中性</t>
         </is>
       </c>
       <c r="C7" s="4" t="inlineStr">
         <is>
-          <t>利空：甘蔗生长阶段的降雨有利于补充土壤水分、改善墒情并促进甘蔗生长和单产形成，从而增加未来甘蔗及食糖供应预期，因此利空糖价。</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="125.75" customHeight="1" s="2">
-      <c r="A8" s="3" t="inlineStr">
-        <is>
-          <t>孟加拉国</t>
-        </is>
-      </c>
-      <c r="B8" s="4" t="inlineStr">
-        <is>
-          <t>孟加拉国糖厂公布乙醇产能、产量或采购价格，披露1.50 lakh。若新增乙醇需求由B重糖蜜、糖浆或甘蔗汁满足，糖厂会把这些可发酵糖源送入乙醇装置；其中B重糖蜜、糖浆和甘蔗汁会减少可结晶成白糖的蔗糖量。来源：Bangladesh Sangbad Sangstha (BSS)（https://www.bssnews.net/district/422685）。影响：利多糖价</t>
-        </is>
-      </c>
-      <c r="C8" s="4" t="inlineStr">
-        <is>
-          <t>利多：若新增乙醇需求由B重糖蜜、糖浆或甘蔗汁满足，糖厂会把这些可发酵糖源送入乙醇装置；其中B重糖蜜、糖浆和甘蔗汁会减少可结晶成白糖的蔗糖量，从而减少食糖供应预期并支撑糖价。</t>
+          <t>中性：基金从净空快速转为净多推高原糖价格，但出口供应仍大、进口需求偏弱限制基本面支撑，涨价影响需要用震荡判断处理。</t>
         </is>
       </c>
     </row>

</xml_diff>